<commit_message>
Scoring calibration, 5-brand fixture rewrite, and UX fixes from debug spec v3
- Recalibrate all 4 scoring functions (ROI, share, volume, inventory) to
  industry benchmarks: breakeven = 55pts, 80%+ net incr = 100pts, healthy
  fill range expanded to 1.08
- Rewrite generate_fixtures.py: 5-brand toothpaste market (15 SKUs), tuned
  pipeline fills (1.08/1.10/1.27), calibrated post-promo factors to produce
  distinct A/B/C grades with correct recommendations
- Fix recommendation ordering so B+Pantry-Loaded fires before B+Moderate inventory
- STAR → STARS in all user-facing text (visualizations, app, ingestion)
- LID tab layout: 2-column split, height=400, metrics in right column

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stella/test_fixtures/inventory_risk/stars_data.xlsx
+++ b/stella/test_fixtures/inventory_risk/stars_data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,23 +485,23 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Whitening 6oz</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>33.9</v>
+        <v>42.79</v>
       </c>
       <c r="E2" t="n">
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>406.76</v>
+        <v>513.48</v>
       </c>
       <c r="G2" t="n">
-        <v>20.41</v>
+        <v>23.25</v>
       </c>
       <c r="H2" t="n">
-        <v>1989.3</v>
+        <v>986.9</v>
       </c>
     </row>
     <row r="3">
@@ -515,28 +515,28 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SF-Variety 12ct</t>
+          <t>SF-Sensitivity 4oz</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>33.39</v>
+        <v>42.98</v>
       </c>
       <c r="E3" t="n">
         <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>400.71</v>
+        <v>515.78</v>
       </c>
       <c r="G3" t="n">
-        <v>19.97</v>
+        <v>23.48</v>
       </c>
       <c r="H3" t="n">
-        <v>1975.9</v>
+        <v>983.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45668</v>
+        <v>45661</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -545,23 +545,23 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Complete 6oz</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>33.92</v>
+        <v>42.63</v>
       </c>
       <c r="E4" t="n">
         <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>407.02</v>
+        <v>511.53</v>
       </c>
       <c r="G4" t="n">
-        <v>20.41</v>
+        <v>23.12</v>
       </c>
       <c r="H4" t="n">
-        <v>1963.3</v>
+        <v>983.4</v>
       </c>
     </row>
     <row r="5">
@@ -575,28 +575,28 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SF-Variety 12ct</t>
+          <t>SF-Whitening 6oz</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>35.24</v>
+        <v>41.73</v>
       </c>
       <c r="E5" t="n">
         <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>422.89</v>
+        <v>500.74</v>
       </c>
       <c r="G5" t="n">
-        <v>21.27</v>
+        <v>22.56</v>
       </c>
       <c r="H5" t="n">
-        <v>1962.8</v>
+        <v>981</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45675</v>
+        <v>45668</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -605,28 +605,28 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Sensitivity 4oz</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>134</v>
+        <v>43.11</v>
       </c>
       <c r="E6" t="n">
         <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>1608</v>
+        <v>517.3099999999999</v>
       </c>
       <c r="G6" t="n">
-        <v>81.31999999999999</v>
+        <v>22.9</v>
       </c>
       <c r="H6" t="n">
-        <v>3084.6</v>
+        <v>963</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45675</v>
+        <v>45668</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -635,28 +635,28 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SF-Variety 12ct</t>
+          <t>SF-Complete 6oz</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>135.25</v>
+        <v>41.55</v>
       </c>
       <c r="E7" t="n">
         <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>1623.05</v>
+        <v>498.65</v>
       </c>
       <c r="G7" t="n">
-        <v>81.56</v>
+        <v>22.65</v>
       </c>
       <c r="H7" t="n">
-        <v>4224.5</v>
+        <v>955.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45682</v>
+        <v>45675</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -665,28 +665,28 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Whitening 6oz</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>136.14</v>
+        <v>192.68</v>
       </c>
       <c r="E8" t="n">
         <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>1633.66</v>
+        <v>2312.16</v>
       </c>
       <c r="G8" t="n">
-        <v>82.45999999999999</v>
+        <v>104.43</v>
       </c>
       <c r="H8" t="n">
-        <v>5380.2</v>
+        <v>2675.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45682</v>
+        <v>45675</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -695,28 +695,28 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SF-Variety 12ct</t>
+          <t>SF-Sensitivity 4oz</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>140.58</v>
+        <v>190.43</v>
       </c>
       <c r="E9" t="n">
         <v>12</v>
       </c>
       <c r="F9" t="n">
-        <v>1686.97</v>
+        <v>2285.13</v>
       </c>
       <c r="G9" t="n">
-        <v>84.36</v>
+        <v>104.33</v>
       </c>
       <c r="H9" t="n">
-        <v>6570.4</v>
+        <v>2650.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45689</v>
+        <v>45675</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -725,28 +725,28 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Complete 6oz</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>69.63</v>
+        <v>191.55</v>
       </c>
       <c r="E10" t="n">
         <v>12</v>
       </c>
       <c r="F10" t="n">
-        <v>835.58</v>
+        <v>2298.63</v>
       </c>
       <c r="G10" t="n">
-        <v>41.47</v>
+        <v>102.89</v>
       </c>
       <c r="H10" t="n">
-        <v>6563.3</v>
+        <v>2642.5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45689</v>
+        <v>45682</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -755,28 +755,28 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SF-Variety 12ct</t>
+          <t>SF-Whitening 6oz</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>67.97</v>
+        <v>185.79</v>
       </c>
       <c r="E11" t="n">
         <v>12</v>
       </c>
       <c r="F11" t="n">
-        <v>815.62</v>
+        <v>2229.46</v>
       </c>
       <c r="G11" t="n">
-        <v>40.15</v>
+        <v>99.09</v>
       </c>
       <c r="H11" t="n">
-        <v>6517.1</v>
+        <v>4324</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>45696</v>
+        <v>45682</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -785,28 +785,28 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Sensitivity 4oz</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>69.86</v>
+        <v>198.05</v>
       </c>
       <c r="E12" t="n">
         <v>12</v>
       </c>
       <c r="F12" t="n">
-        <v>838.33</v>
+        <v>2376.54</v>
       </c>
       <c r="G12" t="n">
-        <v>41.17</v>
+        <v>106.97</v>
       </c>
       <c r="H12" t="n">
-        <v>6541.7</v>
+        <v>4424.9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>45696</v>
+        <v>45682</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -815,28 +815,28 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SF-Variety 12ct</t>
+          <t>SF-Complete 6oz</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>67.09999999999999</v>
+        <v>185.22</v>
       </c>
       <c r="E13" t="n">
         <v>12</v>
       </c>
       <c r="F13" t="n">
-        <v>805.17</v>
+        <v>2222.62</v>
       </c>
       <c r="G13" t="n">
-        <v>39.73</v>
+        <v>99.37</v>
       </c>
       <c r="H13" t="n">
-        <v>6521.2</v>
+        <v>4276.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>45703</v>
+        <v>45689</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -845,28 +845,28 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Whitening 6oz</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>69.31999999999999</v>
+        <v>92.63</v>
       </c>
       <c r="E14" t="n">
         <v>12</v>
       </c>
       <c r="F14" t="n">
-        <v>831.84</v>
+        <v>1111.53</v>
       </c>
       <c r="G14" t="n">
-        <v>40.78</v>
+        <v>50.56</v>
       </c>
       <c r="H14" t="n">
-        <v>6524.1</v>
+        <v>4359.7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>45703</v>
+        <v>45689</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -875,28 +875,28 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SF-Variety 12ct</t>
+          <t>SF-Sensitivity 4oz</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>69.94</v>
+        <v>90.59</v>
       </c>
       <c r="E15" t="n">
         <v>12</v>
       </c>
       <c r="F15" t="n">
-        <v>839.28</v>
+        <v>1087.07</v>
       </c>
       <c r="G15" t="n">
-        <v>41.75</v>
+        <v>49.13</v>
       </c>
       <c r="H15" t="n">
-        <v>6500.7</v>
+        <v>4438.6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>45710</v>
+        <v>45689</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -905,28 +905,28 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Complete 6oz</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>68.55</v>
+        <v>92.77</v>
       </c>
       <c r="E16" t="n">
         <v>12</v>
       </c>
       <c r="F16" t="n">
-        <v>822.58</v>
+        <v>1113.22</v>
       </c>
       <c r="G16" t="n">
-        <v>40.5</v>
+        <v>49.19</v>
       </c>
       <c r="H16" t="n">
-        <v>6505</v>
+        <v>4303.7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>45710</v>
+        <v>45696</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -935,28 +935,28 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SF-Variety 12ct</t>
+          <t>SF-Whitening 6oz</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>70.48999999999999</v>
+        <v>96.37</v>
       </c>
       <c r="E17" t="n">
         <v>12</v>
       </c>
       <c r="F17" t="n">
-        <v>845.9299999999999</v>
+        <v>1156.44</v>
       </c>
       <c r="G17" t="n">
-        <v>43.13</v>
+        <v>52.09</v>
       </c>
       <c r="H17" t="n">
-        <v>6516.4</v>
+        <v>4430.2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>45717</v>
+        <v>45696</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -965,28 +965,28 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Sensitivity 4oz</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>10.05</v>
+        <v>91.34</v>
       </c>
       <c r="E18" t="n">
         <v>12</v>
       </c>
       <c r="F18" t="n">
-        <v>120.55</v>
+        <v>1096.13</v>
       </c>
       <c r="G18" t="n">
-        <v>6.07</v>
+        <v>49.96</v>
       </c>
       <c r="H18" t="n">
-        <v>6303.9</v>
+        <v>4480.6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>45717</v>
+        <v>45696</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -995,28 +995,28 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SF-Variety 12ct</t>
+          <t>SF-Complete 6oz</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>10.11</v>
+        <v>90.01000000000001</v>
       </c>
       <c r="E19" t="n">
         <v>12</v>
       </c>
       <c r="F19" t="n">
-        <v>121.3</v>
+        <v>1080.16</v>
       </c>
       <c r="G19" t="n">
-        <v>6.1</v>
+        <v>48.96</v>
       </c>
       <c r="H19" t="n">
-        <v>6093.8</v>
+        <v>4335</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>45724</v>
+        <v>45703</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1025,28 +1025,28 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Whitening 6oz</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>9.960000000000001</v>
+        <v>95.95999999999999</v>
       </c>
       <c r="E20" t="n">
         <v>12</v>
       </c>
       <c r="F20" t="n">
-        <v>119.55</v>
+        <v>1151.54</v>
       </c>
       <c r="G20" t="n">
-        <v>5.98</v>
+        <v>51.36</v>
       </c>
       <c r="H20" t="n">
-        <v>5899.9</v>
+        <v>4494.4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>45724</v>
+        <v>45703</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1055,28 +1055,28 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SF-Variety 12ct</t>
+          <t>SF-Sensitivity 4oz</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>9.93</v>
+        <v>96.79000000000001</v>
       </c>
       <c r="E21" t="n">
         <v>12</v>
       </c>
       <c r="F21" t="n">
-        <v>119.13</v>
+        <v>1161.53</v>
       </c>
       <c r="G21" t="n">
-        <v>6.04</v>
+        <v>53.18</v>
       </c>
       <c r="H21" t="n">
-        <v>5701.6</v>
+        <v>4624.7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>45731</v>
+        <v>45703</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1085,28 +1085,28 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Complete 6oz</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>10.25</v>
+        <v>94.56</v>
       </c>
       <c r="E22" t="n">
         <v>12</v>
       </c>
       <c r="F22" t="n">
-        <v>122.95</v>
+        <v>1134.77</v>
       </c>
       <c r="G22" t="n">
-        <v>6.23</v>
+        <v>50.99</v>
       </c>
       <c r="H22" t="n">
-        <v>5485.8</v>
+        <v>4416.2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>45731</v>
+        <v>45710</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1115,28 +1115,28 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SF-Variety 12ct</t>
+          <t>SF-Whitening 6oz</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9.91</v>
+        <v>90.65000000000001</v>
       </c>
       <c r="E23" t="n">
         <v>12</v>
       </c>
       <c r="F23" t="n">
-        <v>118.89</v>
+        <v>1087.84</v>
       </c>
       <c r="G23" t="n">
-        <v>5.93</v>
+        <v>48.16</v>
       </c>
       <c r="H23" t="n">
-        <v>5266.2</v>
+        <v>4540.5</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>45738</v>
+        <v>45710</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1145,28 +1145,28 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Sensitivity 4oz</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>9.859999999999999</v>
+        <v>96.02</v>
       </c>
       <c r="E24" t="n">
         <v>12</v>
       </c>
       <c r="F24" t="n">
-        <v>118.29</v>
+        <v>1152.22</v>
       </c>
       <c r="G24" t="n">
-        <v>5.97</v>
+        <v>51.12</v>
       </c>
       <c r="H24" t="n">
-        <v>5061.3</v>
+        <v>4747.1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>45738</v>
+        <v>45710</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1175,28 +1175,28 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SF-Variety 12ct</t>
+          <t>SF-Complete 6oz</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>10.17</v>
+        <v>93.86</v>
       </c>
       <c r="E25" t="n">
         <v>12</v>
       </c>
       <c r="F25" t="n">
-        <v>122.1</v>
+        <v>1126.36</v>
       </c>
       <c r="G25" t="n">
-        <v>6.02</v>
+        <v>50.11</v>
       </c>
       <c r="H25" t="n">
-        <v>4859.1</v>
+        <v>4514.3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>45745</v>
+        <v>45717</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1205,28 +1205,28 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Whitening 6oz</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>24.58</v>
+        <v>12.81</v>
       </c>
       <c r="E26" t="n">
         <v>12</v>
       </c>
       <c r="F26" t="n">
-        <v>294.9</v>
+        <v>153.77</v>
       </c>
       <c r="G26" t="n">
-        <v>14.48</v>
+        <v>6.88</v>
       </c>
       <c r="H26" t="n">
-        <v>4827.7</v>
+        <v>4298.1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>45745</v>
+        <v>45717</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1235,28 +1235,28 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SF-Variety 12ct</t>
+          <t>SF-Sensitivity 4oz</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>23.4</v>
+        <v>13.17</v>
       </c>
       <c r="E27" t="n">
         <v>12</v>
       </c>
       <c r="F27" t="n">
-        <v>280.85</v>
+        <v>158.05</v>
       </c>
       <c r="G27" t="n">
-        <v>14.04</v>
+        <v>7.01</v>
       </c>
       <c r="H27" t="n">
-        <v>4781.3</v>
+        <v>4494.1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>45752</v>
+        <v>45717</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1265,28 +1265,28 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Complete 6oz</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>23.79</v>
+        <v>13.16</v>
       </c>
       <c r="E28" t="n">
         <v>12</v>
       </c>
       <c r="F28" t="n">
-        <v>285.45</v>
+        <v>157.93</v>
       </c>
       <c r="G28" t="n">
-        <v>14.03</v>
+        <v>7.2</v>
       </c>
       <c r="H28" t="n">
-        <v>4730.5</v>
+        <v>4251.8</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>45752</v>
+        <v>45724</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1295,28 +1295,28 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SF-Variety 12ct</t>
+          <t>SF-Whitening 6oz</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>24.45</v>
+        <v>12.87</v>
       </c>
       <c r="E29" t="n">
         <v>12</v>
       </c>
       <c r="F29" t="n">
-        <v>293.45</v>
+        <v>154.47</v>
       </c>
       <c r="G29" t="n">
-        <v>14.75</v>
+        <v>6.99</v>
       </c>
       <c r="H29" t="n">
-        <v>4695.8</v>
+        <v>4031.3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>45759</v>
+        <v>45724</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1325,28 +1325,28 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Sensitivity 4oz</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>24.12</v>
+        <v>12.26</v>
       </c>
       <c r="E30" t="n">
         <v>12</v>
       </c>
       <c r="F30" t="n">
-        <v>289.49</v>
+        <v>147.08</v>
       </c>
       <c r="G30" t="n">
-        <v>14.63</v>
+        <v>6.74</v>
       </c>
       <c r="H30" t="n">
-        <v>4646.8</v>
+        <v>4218.2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>45759</v>
+        <v>45724</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1355,28 +1355,28 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SF-Variety 12ct</t>
+          <t>SF-Complete 6oz</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>23.55</v>
+        <v>13.04</v>
       </c>
       <c r="E31" t="n">
         <v>12</v>
       </c>
       <c r="F31" t="n">
-        <v>282.55</v>
+        <v>156.45</v>
       </c>
       <c r="G31" t="n">
-        <v>14.15</v>
+        <v>7.01</v>
       </c>
       <c r="H31" t="n">
-        <v>4606.5</v>
+        <v>3988.4</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>45766</v>
+        <v>45731</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1385,53 +1385,533 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SF-Original 12ct</t>
+          <t>SF-Whitening 6oz</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>24.46</v>
+        <v>17.01</v>
       </c>
       <c r="E32" t="n">
         <v>12</v>
       </c>
       <c r="F32" t="n">
-        <v>293.47</v>
+        <v>204.16</v>
       </c>
       <c r="G32" t="n">
-        <v>14.66</v>
+        <v>9.19</v>
       </c>
       <c r="H32" t="n">
-        <v>4569.5</v>
+        <v>3822.7</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
+        <v>45731</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>SF-Sensitivity 4oz</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>16.78</v>
+      </c>
+      <c r="E33" t="n">
+        <v>12</v>
+      </c>
+      <c r="F33" t="n">
+        <v>201.38</v>
+      </c>
+      <c r="G33" t="n">
+        <v>8.970000000000001</v>
+      </c>
+      <c r="H33" t="n">
+        <v>3992.8</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>45731</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>SF-Complete 6oz</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>16.83</v>
+      </c>
+      <c r="E34" t="n">
+        <v>12</v>
+      </c>
+      <c r="F34" t="n">
+        <v>201.96</v>
+      </c>
+      <c r="G34" t="n">
+        <v>9.26</v>
+      </c>
+      <c r="H34" t="n">
+        <v>3760.2</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>45738</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>SF-Whitening 6oz</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>16.75</v>
+      </c>
+      <c r="E35" t="n">
+        <v>12</v>
+      </c>
+      <c r="F35" t="n">
+        <v>201.06</v>
+      </c>
+      <c r="G35" t="n">
+        <v>8.970000000000001</v>
+      </c>
+      <c r="H35" t="n">
+        <v>3596</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>45738</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>SF-Sensitivity 4oz</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>17</v>
+      </c>
+      <c r="E36" t="n">
+        <v>12</v>
+      </c>
+      <c r="F36" t="n">
+        <v>203.99</v>
+      </c>
+      <c r="G36" t="n">
+        <v>9.23</v>
+      </c>
+      <c r="H36" t="n">
+        <v>3756</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>45738</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>SF-Complete 6oz</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>16.71</v>
+      </c>
+      <c r="E37" t="n">
+        <v>12</v>
+      </c>
+      <c r="F37" t="n">
+        <v>200.49</v>
+      </c>
+      <c r="G37" t="n">
+        <v>9.09</v>
+      </c>
+      <c r="H37" t="n">
+        <v>3506.1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>45745</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>SF-Whitening 6oz</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="E38" t="n">
+        <v>12</v>
+      </c>
+      <c r="F38" t="n">
+        <v>325.2</v>
+      </c>
+      <c r="G38" t="n">
+        <v>14.61</v>
+      </c>
+      <c r="H38" t="n">
+        <v>3473.7</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>45745</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>SF-Sensitivity 4oz</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>27.89</v>
+      </c>
+      <c r="E39" t="n">
+        <v>12</v>
+      </c>
+      <c r="F39" t="n">
+        <v>334.62</v>
+      </c>
+      <c r="G39" t="n">
+        <v>15.17</v>
+      </c>
+      <c r="H39" t="n">
+        <v>3642.4</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>45745</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>SF-Complete 6oz</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>27.66</v>
+      </c>
+      <c r="E40" t="n">
+        <v>12</v>
+      </c>
+      <c r="F40" t="n">
+        <v>331.94</v>
+      </c>
+      <c r="G40" t="n">
+        <v>15</v>
+      </c>
+      <c r="H40" t="n">
+        <v>3364.2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>45752</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>SF-Whitening 6oz</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>26.61</v>
+      </c>
+      <c r="E41" t="n">
+        <v>12</v>
+      </c>
+      <c r="F41" t="n">
+        <v>319.33</v>
+      </c>
+      <c r="G41" t="n">
+        <v>14.14</v>
+      </c>
+      <c r="H41" t="n">
+        <v>3317.7</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>45752</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>SF-Sensitivity 4oz</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>28.72</v>
+      </c>
+      <c r="E42" t="n">
+        <v>12</v>
+      </c>
+      <c r="F42" t="n">
+        <v>344.64</v>
+      </c>
+      <c r="G42" t="n">
+        <v>15.21</v>
+      </c>
+      <c r="H42" t="n">
+        <v>3501</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>45752</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>SF-Complete 6oz</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>28.18</v>
+      </c>
+      <c r="E43" t="n">
+        <v>12</v>
+      </c>
+      <c r="F43" t="n">
+        <v>338.16</v>
+      </c>
+      <c r="G43" t="n">
+        <v>15.42</v>
+      </c>
+      <c r="H43" t="n">
+        <v>3219.8</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>45759</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>SF-Whitening 6oz</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>27.89</v>
+      </c>
+      <c r="E44" t="n">
+        <v>12</v>
+      </c>
+      <c r="F44" t="n">
+        <v>334.68</v>
+      </c>
+      <c r="G44" t="n">
+        <v>15.18</v>
+      </c>
+      <c r="H44" t="n">
+        <v>3160.5</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>45759</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>SF-Sensitivity 4oz</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>26.79</v>
+      </c>
+      <c r="E45" t="n">
+        <v>12</v>
+      </c>
+      <c r="F45" t="n">
+        <v>321.48</v>
+      </c>
+      <c r="G45" t="n">
+        <v>14.71</v>
+      </c>
+      <c r="H45" t="n">
+        <v>3319.2</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45759</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>SF-Complete 6oz</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>28.37</v>
+      </c>
+      <c r="E46" t="n">
+        <v>12</v>
+      </c>
+      <c r="F46" t="n">
+        <v>340.42</v>
+      </c>
+      <c r="G46" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="H46" t="n">
+        <v>3088.2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
         <v>45766</v>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Summit Foods</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>SF-Variety 12ct</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>24.47</v>
-      </c>
-      <c r="E33" t="n">
-        <v>12</v>
-      </c>
-      <c r="F33" t="n">
-        <v>293.64</v>
-      </c>
-      <c r="G33" t="n">
-        <v>14.68</v>
-      </c>
-      <c r="H33" t="n">
-        <v>4521.6</v>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>SF-Whitening 6oz</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>26.53</v>
+      </c>
+      <c r="E47" t="n">
+        <v>12</v>
+      </c>
+      <c r="F47" t="n">
+        <v>318.34</v>
+      </c>
+      <c r="G47" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="H47" t="n">
+        <v>2976.8</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>45766</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>SF-Sensitivity 4oz</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>26.89</v>
+      </c>
+      <c r="E48" t="n">
+        <v>12</v>
+      </c>
+      <c r="F48" t="n">
+        <v>322.64</v>
+      </c>
+      <c r="G48" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="H48" t="n">
+        <v>3133.9</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>45766</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Summit Foods</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>SF-Complete 6oz</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>28.22</v>
+      </c>
+      <c r="E49" t="n">
+        <v>12</v>
+      </c>
+      <c r="F49" t="n">
+        <v>338.6</v>
+      </c>
+      <c r="G49" t="n">
+        <v>15.48</v>
+      </c>
+      <c r="H49" t="n">
+        <v>2915.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>